<commit_message>
Added progress For october 5
</commit_message>
<xml_diff>
--- a/vaibhav.xlsx
+++ b/vaibhav.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\CAP776\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F3C4FB7-9A6F-4FAF-AB61-95976C636E1E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C56C9B2-4B47-4A99-A6BB-59F8B132D405}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="276" uniqueCount="106">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -193,9 +193,6 @@
     <t>Vaibhav Joshi</t>
   </si>
   <si>
-    <t>MCA Gen</t>
-  </si>
-  <si>
     <t>August</t>
   </si>
   <si>
@@ -247,10 +244,106 @@
     <t>nil</t>
   </si>
   <si>
-    <t>5o</t>
+    <t>Very Unsatisfied</t>
   </si>
   <si>
-    <t>Very Unsatisfied</t>
+    <t>coming back to the college</t>
+  </si>
+  <si>
+    <t>reached early morning</t>
+  </si>
+  <si>
+    <t>packing for the trip back to home</t>
+  </si>
+  <si>
+    <t>enjoying homely vibes and food</t>
+  </si>
+  <si>
+    <t>celebrating rakshabandhan at home</t>
+  </si>
+  <si>
+    <t>MCA General</t>
+  </si>
+  <si>
+    <t>python class was cancelled</t>
+  </si>
+  <si>
+    <t>gave DCN CA-1</t>
+  </si>
+  <si>
+    <t>enjoyed our fresher's party</t>
+  </si>
+  <si>
+    <t>had a very relaxing and soothing day. All the stress and tiredness was gone.</t>
+  </si>
+  <si>
+    <t>cleaned the room today</t>
+  </si>
+  <si>
+    <t>washed all dirty clothes today</t>
+  </si>
+  <si>
+    <t>washed my shoes today</t>
+  </si>
+  <si>
+    <t>nothing special happened today</t>
+  </si>
+  <si>
+    <t>had a stressfree day today</t>
+  </si>
+  <si>
+    <t>fasting on the occasion of janmasthami</t>
+  </si>
+  <si>
+    <t>not well today</t>
+  </si>
+  <si>
+    <t>purchasing stuff for my trip</t>
+  </si>
+  <si>
+    <t>packing for the journey</t>
+  </si>
+  <si>
+    <t>reached back late at night</t>
+  </si>
+  <si>
+    <t>started my journey at night</t>
+  </si>
+  <si>
+    <t>day 1 of trip</t>
+  </si>
+  <si>
+    <t>day 2 of trip</t>
+  </si>
+  <si>
+    <t>day 3 of trip</t>
+  </si>
+  <si>
+    <t>day 4 of trip</t>
+  </si>
+  <si>
+    <t>way back to college</t>
+  </si>
+  <si>
+    <t>exhausted</t>
+  </si>
+  <si>
+    <t xml:space="preserve">preaparing for the CA exam </t>
+  </si>
+  <si>
+    <t xml:space="preserve">gave communication CA exam </t>
+  </si>
+  <si>
+    <t>college closed from today till next 10 days due to the protest/riot</t>
+  </si>
+  <si>
+    <t>riot broke down in the college campus at midnight</t>
+  </si>
+  <si>
+    <t>watched a movie today</t>
+  </si>
+  <si>
+    <t>gave dbms CA1</t>
   </si>
 </sst>
 </file>
@@ -955,7 +1048,7 @@
         <v>32</v>
       </c>
       <c r="B3" s="20" t="s">
-        <v>55</v>
+        <v>78</v>
       </c>
       <c r="C3" s="20"/>
       <c r="D3" s="20"/>
@@ -963,7 +1056,7 @@
         <v>33</v>
       </c>
       <c r="F3" s="20" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G3" s="20"/>
     </row>
@@ -1109,16 +1202,16 @@
         <v>550</v>
       </c>
       <c r="K7" s="16" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="L7" s="16" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="M7" s="16" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="N7" s="17" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="8" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
@@ -1155,16 +1248,16 @@
         <v>410</v>
       </c>
       <c r="K8" s="16" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="L8" s="16" t="s">
         <v>50</v>
       </c>
       <c r="M8" s="16" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="N8" s="17" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="9" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
@@ -1187,7 +1280,7 @@
         <v>430</v>
       </c>
       <c r="G9" s="14" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="H9" s="14">
         <v>60</v>
@@ -1201,16 +1294,16 @@
         <v>370</v>
       </c>
       <c r="K9" s="16" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="L9" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="M9" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="M9" s="16" t="s">
-        <v>58</v>
-      </c>
       <c r="N9" s="17" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.3">
@@ -1247,21 +1340,21 @@
         <v>360</v>
       </c>
       <c r="K10" s="16" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="L10" s="16" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="M10" s="16" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="N10" s="17" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A11" s="13" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B11" s="14">
         <v>440</v>
@@ -1293,15 +1386,17 @@
         <v>470</v>
       </c>
       <c r="K11" s="16" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="L11" s="16" t="s">
         <v>50</v>
       </c>
       <c r="M11" s="16" t="s">
-        <v>59</v>
-      </c>
-      <c r="N11" s="17"/>
+        <v>58</v>
+      </c>
+      <c r="N11" s="17" t="s">
+        <v>87</v>
+      </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A12" s="13">
@@ -1320,10 +1415,10 @@
         <v>120</v>
       </c>
       <c r="F12" s="14" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="G12" s="14" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="H12" s="14">
         <v>180</v>
@@ -1337,15 +1432,17 @@
         <v>290</v>
       </c>
       <c r="K12" s="16" t="s">
+        <v>63</v>
+      </c>
+      <c r="L12" s="16" t="s">
         <v>64</v>
-      </c>
-      <c r="L12" s="16" t="s">
-        <v>65</v>
       </c>
       <c r="M12" s="16" t="s">
         <v>51</v>
       </c>
-      <c r="N12" s="17"/>
+      <c r="N12" s="17" t="s">
+        <v>84</v>
+      </c>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A13" s="13">
@@ -1364,10 +1461,10 @@
         <v>70</v>
       </c>
       <c r="F13" s="14" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="G13" s="14" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="H13" s="14">
         <v>240</v>
@@ -1381,15 +1478,17 @@
         <v>240</v>
       </c>
       <c r="K13" s="16" t="s">
+        <v>63</v>
+      </c>
+      <c r="L13" s="16" t="s">
         <v>64</v>
-      </c>
-      <c r="L13" s="16" t="s">
-        <v>65</v>
       </c>
       <c r="M13" s="16" t="s">
         <v>51</v>
       </c>
-      <c r="N13" s="17"/>
+      <c r="N13" s="17" t="s">
+        <v>85</v>
+      </c>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A14" s="13">
@@ -1413,25 +1512,25 @@
       <c r="G14" s="14">
         <v>6</v>
       </c>
-      <c r="H14" s="14" t="s">
-        <v>73</v>
+      <c r="H14" s="14">
+        <v>50</v>
       </c>
       <c r="I14" s="15">
         <f t="shared" si="0"/>
-        <v>825</v>
+        <v>875</v>
       </c>
       <c r="J14" s="15">
         <f t="shared" si="1"/>
-        <v>615</v>
+        <v>565</v>
       </c>
       <c r="K14" s="16" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="L14" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="M14" s="16" t="s">
         <v>57</v>
-      </c>
-      <c r="M14" s="16" t="s">
-        <v>58</v>
       </c>
       <c r="N14" s="17"/>
     </row>
@@ -1469,13 +1568,13 @@
         <v>760</v>
       </c>
       <c r="K15" s="16" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="L15" s="16" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="M15" s="16" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="N15" s="17"/>
     </row>
@@ -1483,924 +1582,1880 @@
       <c r="A16" s="13">
         <v>46253</v>
       </c>
-      <c r="B16" s="14"/>
-      <c r="C16" s="14"/>
-      <c r="D16" s="14"/>
-      <c r="E16" s="14"/>
-      <c r="F16" s="14"/>
+      <c r="B16" s="14">
+        <v>340</v>
+      </c>
+      <c r="C16" s="14">
+        <v>0</v>
+      </c>
+      <c r="D16" s="14">
+        <v>120</v>
+      </c>
+      <c r="E16" s="14">
+        <v>30</v>
+      </c>
+      <c r="F16" s="14">
+        <v>350</v>
+      </c>
       <c r="G16" s="14">
         <v>7</v>
       </c>
-      <c r="H16" s="14"/>
-      <c r="I16" s="15" t="str">
+      <c r="H16" s="14">
+        <v>85</v>
+      </c>
+      <c r="I16" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J16" s="15" t="str">
+        <v>925</v>
+      </c>
+      <c r="J16" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K16" s="16"/>
-      <c r="L16" s="16"/>
-      <c r="M16" s="16"/>
+        <v>515</v>
+      </c>
+      <c r="K16" s="16" t="s">
+        <v>60</v>
+      </c>
+      <c r="L16" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="M16" s="16" t="s">
+        <v>57</v>
+      </c>
       <c r="N16" s="17"/>
     </row>
     <row r="17" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A17" s="13">
         <v>46254</v>
       </c>
-      <c r="B17" s="14"/>
-      <c r="C17" s="14"/>
-      <c r="D17" s="14"/>
-      <c r="E17" s="14"/>
-      <c r="F17" s="14"/>
+      <c r="B17" s="14">
+        <v>390</v>
+      </c>
+      <c r="C17" s="14">
+        <v>10</v>
+      </c>
+      <c r="D17" s="14">
+        <v>140</v>
+      </c>
+      <c r="E17" s="14">
+        <v>50</v>
+      </c>
+      <c r="F17" s="14">
+        <v>150</v>
+      </c>
       <c r="G17" s="14">
         <v>3</v>
       </c>
-      <c r="H17" s="14"/>
-      <c r="I17" s="15" t="str">
+      <c r="H17" s="14">
+        <v>200</v>
+      </c>
+      <c r="I17" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J17" s="15" t="str">
+        <v>940</v>
+      </c>
+      <c r="J17" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K17" s="16"/>
-      <c r="L17" s="16"/>
-      <c r="M17" s="16"/>
+        <v>500</v>
+      </c>
+      <c r="K17" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="L17" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="M17" s="16" t="s">
+        <v>58</v>
+      </c>
       <c r="N17" s="17"/>
     </row>
     <row r="18" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A18" s="13">
         <v>46255</v>
       </c>
-      <c r="B18" s="14"/>
-      <c r="C18" s="14"/>
-      <c r="D18" s="14"/>
-      <c r="E18" s="14"/>
-      <c r="F18" s="14"/>
+      <c r="B18" s="14">
+        <v>280</v>
+      </c>
+      <c r="C18" s="14">
+        <v>10</v>
+      </c>
+      <c r="D18" s="14">
+        <v>50</v>
+      </c>
+      <c r="E18" s="14">
+        <v>110</v>
+      </c>
+      <c r="F18" s="14">
+        <v>200</v>
+      </c>
       <c r="G18" s="14">
         <v>4</v>
       </c>
-      <c r="H18" s="14"/>
-      <c r="I18" s="15" t="str">
+      <c r="H18" s="14">
+        <v>200</v>
+      </c>
+      <c r="I18" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J18" s="15" t="str">
+        <v>850</v>
+      </c>
+      <c r="J18" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K18" s="16"/>
-      <c r="L18" s="16"/>
-      <c r="M18" s="16"/>
-      <c r="N18" s="17"/>
-    </row>
-    <row r="19" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A19" s="13"/>
-      <c r="B19" s="14"/>
-      <c r="C19" s="14"/>
-      <c r="D19" s="14"/>
-      <c r="E19" s="14"/>
-      <c r="F19" s="14"/>
-      <c r="G19" s="14"/>
-      <c r="H19" s="14"/>
-      <c r="I19" s="15" t="str">
+        <v>590</v>
+      </c>
+      <c r="K18" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="L18" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M18" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="N18" s="17" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="19" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A19" s="13">
+        <v>46256</v>
+      </c>
+      <c r="B19" s="14">
+        <v>560</v>
+      </c>
+      <c r="C19" s="14">
+        <v>20</v>
+      </c>
+      <c r="D19" s="14">
+        <v>120</v>
+      </c>
+      <c r="E19" s="14">
+        <v>50</v>
+      </c>
+      <c r="F19" s="14" t="s">
+        <v>71</v>
+      </c>
+      <c r="G19" s="14" t="s">
+        <v>68</v>
+      </c>
+      <c r="H19" s="14">
+        <v>240</v>
+      </c>
+      <c r="I19" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J19" s="15" t="str">
+        <v>990</v>
+      </c>
+      <c r="J19" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K19" s="16"/>
-      <c r="L19" s="16"/>
-      <c r="M19" s="16"/>
-      <c r="N19" s="17"/>
+        <v>450</v>
+      </c>
+      <c r="K19" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L19" s="16" t="s">
+        <v>64</v>
+      </c>
+      <c r="M19" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="N19" s="17" t="s">
+        <v>82</v>
+      </c>
     </row>
     <row r="20" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A20" s="13"/>
-      <c r="B20" s="14"/>
-      <c r="C20" s="14"/>
-      <c r="D20" s="14"/>
-      <c r="E20" s="14"/>
-      <c r="F20" s="14"/>
-      <c r="G20" s="14"/>
-      <c r="H20" s="14"/>
-      <c r="I20" s="15" t="str">
+      <c r="A20" s="13">
+        <v>46257</v>
+      </c>
+      <c r="B20" s="14">
+        <v>550</v>
+      </c>
+      <c r="C20" s="14">
+        <v>30</v>
+      </c>
+      <c r="D20" s="14">
+        <v>180</v>
+      </c>
+      <c r="E20" s="14">
+        <v>70</v>
+      </c>
+      <c r="F20" s="14" t="s">
+        <v>71</v>
+      </c>
+      <c r="G20" s="14" t="s">
+        <v>69</v>
+      </c>
+      <c r="H20" s="14">
+        <v>280</v>
+      </c>
+      <c r="I20" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J20" s="15" t="str">
+        <v>1110</v>
+      </c>
+      <c r="J20" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K20" s="16"/>
-      <c r="L20" s="16"/>
-      <c r="M20" s="16"/>
-      <c r="N20" s="17"/>
+        <v>330</v>
+      </c>
+      <c r="K20" s="16" t="s">
+        <v>63</v>
+      </c>
+      <c r="L20" s="16" t="s">
+        <v>64</v>
+      </c>
+      <c r="M20" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="N20" s="17" t="s">
+        <v>83</v>
+      </c>
     </row>
     <row r="21" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A21" s="13"/>
-      <c r="B21" s="14"/>
-      <c r="C21" s="14"/>
-      <c r="D21" s="14"/>
-      <c r="E21" s="14"/>
-      <c r="F21" s="14"/>
-      <c r="G21" s="14"/>
-      <c r="H21" s="14"/>
-      <c r="I21" s="15" t="str">
+      <c r="A21" s="13">
+        <v>46258</v>
+      </c>
+      <c r="B21" s="14">
+        <v>360</v>
+      </c>
+      <c r="C21" s="14">
+        <v>30</v>
+      </c>
+      <c r="D21" s="14">
+        <v>255</v>
+      </c>
+      <c r="E21" s="14">
+        <v>45</v>
+      </c>
+      <c r="F21" s="14">
+        <v>250</v>
+      </c>
+      <c r="G21" s="14">
+        <v>5</v>
+      </c>
+      <c r="H21" s="14">
+        <v>250</v>
+      </c>
+      <c r="I21" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J21" s="15" t="str">
+        <v>1190</v>
+      </c>
+      <c r="J21" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K21" s="16"/>
-      <c r="L21" s="16"/>
-      <c r="M21" s="16"/>
+        <v>250</v>
+      </c>
+      <c r="K21" s="16" t="s">
+        <v>63</v>
+      </c>
+      <c r="L21" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M21" s="16" t="s">
+        <v>51</v>
+      </c>
       <c r="N21" s="17"/>
     </row>
     <row r="22" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A22" s="13"/>
-      <c r="B22" s="14"/>
-      <c r="C22" s="14"/>
-      <c r="D22" s="14"/>
-      <c r="E22" s="14"/>
-      <c r="F22" s="14"/>
-      <c r="G22" s="14"/>
-      <c r="H22" s="14"/>
-      <c r="I22" s="15" t="str">
+      <c r="A22" s="13">
+        <v>46259</v>
+      </c>
+      <c r="B22" s="14">
+        <v>400</v>
+      </c>
+      <c r="C22" s="14">
+        <v>0</v>
+      </c>
+      <c r="D22" s="14">
+        <v>30</v>
+      </c>
+      <c r="E22" s="14">
+        <v>180</v>
+      </c>
+      <c r="F22" s="14">
+        <v>350</v>
+      </c>
+      <c r="G22" s="14">
+        <v>7</v>
+      </c>
+      <c r="H22" s="14">
+        <v>100</v>
+      </c>
+      <c r="I22" s="15">
+        <f>J28</f>
+        <v>570</v>
+      </c>
+      <c r="J22" s="15">
+        <f t="shared" si="1"/>
+        <v>870</v>
+      </c>
+      <c r="K22" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L22" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="M22" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="N22" s="17"/>
+    </row>
+    <row r="23" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A23" s="13">
+        <v>46260</v>
+      </c>
+      <c r="B23" s="14">
+        <v>295</v>
+      </c>
+      <c r="C23" s="14">
+        <v>20</v>
+      </c>
+      <c r="D23" s="14">
+        <v>60</v>
+      </c>
+      <c r="E23" s="14">
+        <v>100</v>
+      </c>
+      <c r="F23" s="14">
+        <v>300</v>
+      </c>
+      <c r="G23" s="14">
+        <v>6</v>
+      </c>
+      <c r="H23" s="14">
+        <v>275</v>
+      </c>
+      <c r="I23" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J22" s="15" t="str">
+        <v>1050</v>
+      </c>
+      <c r="J23" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K22" s="16"/>
-      <c r="L22" s="16"/>
-      <c r="M22" s="16"/>
-      <c r="N22" s="17"/>
-    </row>
-    <row r="23" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A23" s="13"/>
-      <c r="B23" s="14"/>
-      <c r="C23" s="14"/>
-      <c r="D23" s="14"/>
-      <c r="E23" s="14"/>
-      <c r="F23" s="14"/>
-      <c r="G23" s="14"/>
-      <c r="H23" s="14"/>
-      <c r="I23" s="15" t="str">
+        <v>390</v>
+      </c>
+      <c r="K23" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="L23" s="16" t="s">
+        <v>72</v>
+      </c>
+      <c r="M23" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="N23" s="17"/>
+    </row>
+    <row r="24" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A24" s="13">
+        <v>46261</v>
+      </c>
+      <c r="B24" s="14">
+        <v>380</v>
+      </c>
+      <c r="C24" s="14">
+        <v>30</v>
+      </c>
+      <c r="D24" s="14">
+        <v>95</v>
+      </c>
+      <c r="E24" s="14">
+        <v>50</v>
+      </c>
+      <c r="F24" s="14">
+        <v>150</v>
+      </c>
+      <c r="G24" s="14">
+        <v>3</v>
+      </c>
+      <c r="H24" s="14">
+        <v>350</v>
+      </c>
+      <c r="I24" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J23" s="15" t="str">
+        <v>1055</v>
+      </c>
+      <c r="J24" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K23" s="16"/>
-      <c r="L23" s="16"/>
-      <c r="M23" s="16"/>
-      <c r="N23" s="17"/>
-    </row>
-    <row r="24" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A24" s="13"/>
-      <c r="B24" s="14"/>
-      <c r="C24" s="14"/>
-      <c r="D24" s="14"/>
-      <c r="E24" s="14"/>
-      <c r="F24" s="14"/>
-      <c r="G24" s="14"/>
-      <c r="H24" s="14"/>
-      <c r="I24" s="15" t="str">
+        <v>385</v>
+      </c>
+      <c r="K24" s="16" t="s">
+        <v>63</v>
+      </c>
+      <c r="L24" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="M24" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="N24" s="17" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="25" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A25" s="13">
+        <v>46262</v>
+      </c>
+      <c r="B25" s="14">
+        <v>440</v>
+      </c>
+      <c r="C25" s="14">
+        <v>0</v>
+      </c>
+      <c r="D25" s="14">
+        <v>0</v>
+      </c>
+      <c r="E25" s="14">
+        <v>0</v>
+      </c>
+      <c r="F25" s="14">
+        <v>0</v>
+      </c>
+      <c r="G25" s="14" t="s">
+        <v>71</v>
+      </c>
+      <c r="H25" s="14">
+        <v>480</v>
+      </c>
+      <c r="I25" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J24" s="15" t="str">
+        <v>920</v>
+      </c>
+      <c r="J25" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K24" s="16"/>
-      <c r="L24" s="16"/>
-      <c r="M24" s="16"/>
-      <c r="N24" s="17"/>
-    </row>
-    <row r="25" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A25" s="13"/>
-      <c r="B25" s="14"/>
-      <c r="C25" s="14"/>
-      <c r="D25" s="14"/>
-      <c r="E25" s="14"/>
-      <c r="F25" s="14"/>
-      <c r="G25" s="14"/>
-      <c r="H25" s="14"/>
-      <c r="I25" s="15" t="str">
+        <v>520</v>
+      </c>
+      <c r="K25" s="16" t="s">
+        <v>63</v>
+      </c>
+      <c r="L25" s="16" t="s">
+        <v>64</v>
+      </c>
+      <c r="M25" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="N25" s="17" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="26" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A26" s="13">
+        <v>46263</v>
+      </c>
+      <c r="B26" s="14">
+        <v>420</v>
+      </c>
+      <c r="C26" s="14">
+        <v>0</v>
+      </c>
+      <c r="D26" s="14">
+        <v>180</v>
+      </c>
+      <c r="E26" s="14">
+        <v>0</v>
+      </c>
+      <c r="F26" s="14" t="s">
+        <v>71</v>
+      </c>
+      <c r="G26" s="14" t="s">
+        <v>68</v>
+      </c>
+      <c r="H26" s="14">
+        <v>300</v>
+      </c>
+      <c r="I26" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J25" s="15" t="str">
+        <v>900</v>
+      </c>
+      <c r="J26" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K25" s="16"/>
-      <c r="L25" s="16"/>
-      <c r="M25" s="16"/>
-      <c r="N25" s="17"/>
-    </row>
-    <row r="26" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A26" s="13"/>
-      <c r="B26" s="14"/>
-      <c r="C26" s="14"/>
-      <c r="D26" s="14"/>
-      <c r="E26" s="14"/>
-      <c r="F26" s="14"/>
-      <c r="G26" s="14"/>
-      <c r="H26" s="14"/>
-      <c r="I26" s="15" t="str">
+        <v>540</v>
+      </c>
+      <c r="K26" s="16" t="s">
+        <v>63</v>
+      </c>
+      <c r="L26" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M26" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="N26" s="17" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="27" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A27" s="13">
+        <v>46264</v>
+      </c>
+      <c r="B27" s="14">
+        <v>435</v>
+      </c>
+      <c r="C27" s="14">
+        <v>0</v>
+      </c>
+      <c r="D27" s="14">
+        <v>120</v>
+      </c>
+      <c r="E27" s="14">
+        <v>0</v>
+      </c>
+      <c r="F27" s="14" t="s">
+        <v>71</v>
+      </c>
+      <c r="G27" s="14" t="s">
+        <v>69</v>
+      </c>
+      <c r="H27" s="14">
+        <v>360</v>
+      </c>
+      <c r="I27" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J26" s="15" t="str">
+        <v>915</v>
+      </c>
+      <c r="J27" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K26" s="16"/>
-      <c r="L26" s="16"/>
-      <c r="M26" s="16"/>
-      <c r="N26" s="17"/>
-    </row>
-    <row r="27" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A27" s="13"/>
-      <c r="B27" s="14"/>
-      <c r="C27" s="14"/>
-      <c r="D27" s="14"/>
-      <c r="E27" s="14"/>
-      <c r="F27" s="14"/>
-      <c r="G27" s="14"/>
-      <c r="H27" s="14"/>
-      <c r="I27" s="15" t="str">
+        <v>525</v>
+      </c>
+      <c r="K27" s="16" t="s">
+        <v>63</v>
+      </c>
+      <c r="L27" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M27" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="N27" s="17" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="28" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A28" s="13">
+        <v>46265</v>
+      </c>
+      <c r="B28" s="14">
+        <v>210</v>
+      </c>
+      <c r="C28" s="14">
+        <v>0</v>
+      </c>
+      <c r="D28" s="14">
+        <v>150</v>
+      </c>
+      <c r="E28" s="14">
+        <v>30</v>
+      </c>
+      <c r="F28" s="14">
+        <v>300</v>
+      </c>
+      <c r="G28" s="14">
+        <v>6</v>
+      </c>
+      <c r="H28" s="14">
+        <v>180</v>
+      </c>
+      <c r="I28" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J27" s="15" t="str">
+        <v>870</v>
+      </c>
+      <c r="J28" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K27" s="16"/>
-      <c r="L27" s="16"/>
-      <c r="M27" s="16"/>
-      <c r="N27" s="17"/>
-    </row>
-    <row r="28" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A28" s="13"/>
-      <c r="B28" s="14"/>
-      <c r="C28" s="14"/>
-      <c r="D28" s="14"/>
-      <c r="E28" s="14"/>
-      <c r="F28" s="14"/>
-      <c r="G28" s="14"/>
-      <c r="H28" s="14"/>
-      <c r="I28" s="15" t="str">
+        <v>570</v>
+      </c>
+      <c r="K28" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="L28" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="M28" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="N28" s="17" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="29" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A29" s="13">
+        <v>46266</v>
+      </c>
+      <c r="B29" s="14">
+        <v>410</v>
+      </c>
+      <c r="C29" s="14">
+        <v>20</v>
+      </c>
+      <c r="D29" s="14">
+        <v>180</v>
+      </c>
+      <c r="E29" s="14">
+        <v>0</v>
+      </c>
+      <c r="F29" s="14">
+        <v>350</v>
+      </c>
+      <c r="G29" s="14">
+        <v>7</v>
+      </c>
+      <c r="H29" s="14">
+        <v>250</v>
+      </c>
+      <c r="I29" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J28" s="15" t="str">
+        <v>1210</v>
+      </c>
+      <c r="J29" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K28" s="16"/>
-      <c r="L28" s="16"/>
-      <c r="M28" s="16"/>
-      <c r="N28" s="17"/>
-    </row>
-    <row r="29" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A29" s="13"/>
-      <c r="B29" s="14"/>
-      <c r="C29" s="14"/>
-      <c r="D29" s="14"/>
-      <c r="E29" s="14"/>
-      <c r="F29" s="14"/>
-      <c r="G29" s="14"/>
-      <c r="H29" s="14"/>
-      <c r="I29" s="15" t="str">
+        <v>230</v>
+      </c>
+      <c r="K29" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="L29" s="16" t="s">
+        <v>72</v>
+      </c>
+      <c r="M29" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N29" s="17" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="30" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A30" s="13">
+        <v>46267</v>
+      </c>
+      <c r="B30" s="14">
+        <v>440</v>
+      </c>
+      <c r="C30" s="14">
+        <v>0</v>
+      </c>
+      <c r="D30" s="14">
+        <v>180</v>
+      </c>
+      <c r="E30" s="14">
+        <v>30</v>
+      </c>
+      <c r="F30" s="14">
+        <v>350</v>
+      </c>
+      <c r="G30" s="14">
+        <v>7</v>
+      </c>
+      <c r="H30" s="14">
+        <v>300</v>
+      </c>
+      <c r="I30" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J29" s="15" t="str">
+        <v>1300</v>
+      </c>
+      <c r="J30" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K29" s="16"/>
-      <c r="L29" s="16"/>
-      <c r="M29" s="16"/>
-      <c r="N29" s="17"/>
-    </row>
-    <row r="30" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A30" s="13"/>
-      <c r="B30" s="14"/>
-      <c r="C30" s="14"/>
-      <c r="D30" s="14"/>
-      <c r="E30" s="14"/>
-      <c r="F30" s="14"/>
-      <c r="G30" s="14"/>
-      <c r="H30" s="14"/>
-      <c r="I30" s="15" t="str">
+        <v>140</v>
+      </c>
+      <c r="K30" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="L30" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="M30" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="N30" s="17" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="31" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A31" s="13">
+        <v>46268</v>
+      </c>
+      <c r="B31" s="14">
+        <v>375</v>
+      </c>
+      <c r="C31" s="14">
+        <v>0</v>
+      </c>
+      <c r="D31" s="14">
+        <v>120</v>
+      </c>
+      <c r="E31" s="14">
+        <v>0</v>
+      </c>
+      <c r="F31" s="14">
+        <v>250</v>
+      </c>
+      <c r="G31" s="14">
+        <v>5</v>
+      </c>
+      <c r="H31" s="14">
+        <v>295</v>
+      </c>
+      <c r="I31" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J30" s="15" t="str">
+        <v>1040</v>
+      </c>
+      <c r="J31" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K30" s="16"/>
-      <c r="L30" s="16"/>
-      <c r="M30" s="16"/>
-      <c r="N30" s="17"/>
-    </row>
-    <row r="31" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A31" s="13"/>
-      <c r="B31" s="14"/>
-      <c r="C31" s="14"/>
-      <c r="D31" s="14"/>
-      <c r="E31" s="14"/>
-      <c r="F31" s="14"/>
-      <c r="G31" s="14"/>
-      <c r="H31" s="14"/>
-      <c r="I31" s="15" t="str">
+        <v>400</v>
+      </c>
+      <c r="K31" s="16" t="s">
+        <v>63</v>
+      </c>
+      <c r="L31" s="16" t="s">
+        <v>64</v>
+      </c>
+      <c r="M31" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="N31" s="17" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="32" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A32" s="13">
+        <v>46269</v>
+      </c>
+      <c r="B32" s="14">
+        <v>270</v>
+      </c>
+      <c r="C32" s="14">
+        <v>0</v>
+      </c>
+      <c r="D32" s="14">
+        <v>180</v>
+      </c>
+      <c r="E32" s="14">
+        <v>70</v>
+      </c>
+      <c r="F32" s="14">
+        <v>300</v>
+      </c>
+      <c r="G32" s="14">
+        <v>6</v>
+      </c>
+      <c r="H32" s="14">
+        <v>150</v>
+      </c>
+      <c r="I32" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J31" s="15" t="str">
+        <v>970</v>
+      </c>
+      <c r="J32" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K31" s="16"/>
-      <c r="L31" s="16"/>
-      <c r="M31" s="16"/>
-      <c r="N31" s="17"/>
-    </row>
-    <row r="32" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A32" s="13"/>
-      <c r="B32" s="14"/>
-      <c r="C32" s="14"/>
-      <c r="D32" s="14"/>
-      <c r="E32" s="14"/>
-      <c r="F32" s="14"/>
-      <c r="G32" s="14"/>
-      <c r="H32" s="14"/>
-      <c r="I32" s="15" t="str">
+        <v>470</v>
+      </c>
+      <c r="K32" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="L32" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M32" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N32" s="17" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="33" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A33" s="13">
+        <v>46270</v>
+      </c>
+      <c r="B33" s="14">
+        <v>500</v>
+      </c>
+      <c r="C33" s="14">
+        <v>30</v>
+      </c>
+      <c r="D33" s="14">
+        <v>200</v>
+      </c>
+      <c r="E33" s="14">
+        <v>120</v>
+      </c>
+      <c r="F33" s="14" t="s">
+        <v>71</v>
+      </c>
+      <c r="G33" s="14" t="s">
+        <v>68</v>
+      </c>
+      <c r="H33" s="14">
+        <v>300</v>
+      </c>
+      <c r="I33" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J32" s="15" t="str">
+        <v>1150</v>
+      </c>
+      <c r="J33" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K32" s="16"/>
-      <c r="L32" s="16"/>
-      <c r="M32" s="16"/>
-      <c r="N32" s="17"/>
-    </row>
-    <row r="33" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A33" s="13"/>
-      <c r="B33" s="14"/>
-      <c r="C33" s="14"/>
-      <c r="D33" s="14"/>
-      <c r="E33" s="14"/>
-      <c r="F33" s="14"/>
-      <c r="G33" s="14"/>
-      <c r="H33" s="14"/>
-      <c r="I33" s="15" t="str">
+        <v>290</v>
+      </c>
+      <c r="K33" s="16" t="s">
+        <v>63</v>
+      </c>
+      <c r="L33" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M33" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="N33" s="17"/>
+    </row>
+    <row r="34" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A34" s="13">
+        <v>46271</v>
+      </c>
+      <c r="B34" s="14">
+        <v>470</v>
+      </c>
+      <c r="C34" s="14">
+        <v>40</v>
+      </c>
+      <c r="D34" s="14">
+        <v>50</v>
+      </c>
+      <c r="E34" s="14">
+        <v>180</v>
+      </c>
+      <c r="F34" s="14" t="s">
+        <v>71</v>
+      </c>
+      <c r="G34" s="14" t="s">
+        <v>69</v>
+      </c>
+      <c r="H34" s="14">
+        <v>350</v>
+      </c>
+      <c r="I34" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J33" s="15" t="str">
+        <v>1090</v>
+      </c>
+      <c r="J34" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K33" s="16"/>
-      <c r="L33" s="16"/>
-      <c r="M33" s="16"/>
-      <c r="N33" s="17"/>
-    </row>
-    <row r="34" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A34" s="13"/>
-      <c r="B34" s="14"/>
-      <c r="C34" s="14"/>
-      <c r="D34" s="14"/>
-      <c r="E34" s="14"/>
-      <c r="F34" s="14"/>
-      <c r="G34" s="14"/>
-      <c r="H34" s="14"/>
-      <c r="I34" s="15" t="str">
+        <v>350</v>
+      </c>
+      <c r="K34" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L34" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="M34" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N34" s="17" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="35" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A35" s="13">
+        <v>46272</v>
+      </c>
+      <c r="B35" s="14">
+        <v>240</v>
+      </c>
+      <c r="C35" s="14">
+        <v>0</v>
+      </c>
+      <c r="D35" s="14">
+        <v>120</v>
+      </c>
+      <c r="E35" s="14">
+        <v>90</v>
+      </c>
+      <c r="F35" s="14">
+        <v>300</v>
+      </c>
+      <c r="G35" s="14">
+        <v>6</v>
+      </c>
+      <c r="H35" s="14">
+        <v>240</v>
+      </c>
+      <c r="I35" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J34" s="15" t="str">
+        <v>990</v>
+      </c>
+      <c r="J35" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K34" s="16"/>
-      <c r="L34" s="16"/>
-      <c r="M34" s="16"/>
-      <c r="N34" s="17"/>
-    </row>
-    <row r="35" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A35" s="13"/>
-      <c r="B35" s="14"/>
-      <c r="C35" s="14"/>
-      <c r="D35" s="14"/>
-      <c r="E35" s="14"/>
-      <c r="F35" s="14"/>
-      <c r="G35" s="14"/>
-      <c r="H35" s="14"/>
-      <c r="I35" s="15" t="str">
+        <v>450</v>
+      </c>
+      <c r="K35" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L35" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M35" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="N35" s="17" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="36" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A36" s="13">
+        <v>46273</v>
+      </c>
+      <c r="B36" s="14">
+        <v>390</v>
+      </c>
+      <c r="C36" s="14">
+        <v>20</v>
+      </c>
+      <c r="D36" s="14">
+        <v>100</v>
+      </c>
+      <c r="E36" s="14">
+        <v>50</v>
+      </c>
+      <c r="F36" s="14">
+        <v>350</v>
+      </c>
+      <c r="G36" s="14">
+        <v>7</v>
+      </c>
+      <c r="H36" s="14">
+        <v>140</v>
+      </c>
+      <c r="I36" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J35" s="15" t="str">
+        <v>1050</v>
+      </c>
+      <c r="J36" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K35" s="16"/>
-      <c r="L35" s="16"/>
-      <c r="M35" s="16"/>
-      <c r="N35" s="17"/>
-    </row>
-    <row r="36" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A36" s="13"/>
-      <c r="B36" s="14"/>
-      <c r="C36" s="14"/>
-      <c r="D36" s="14"/>
-      <c r="E36" s="14"/>
-      <c r="F36" s="14"/>
-      <c r="G36" s="14"/>
-      <c r="H36" s="14"/>
-      <c r="I36" s="15" t="str">
+        <v>390</v>
+      </c>
+      <c r="K36" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="L36" s="16" t="s">
+        <v>72</v>
+      </c>
+      <c r="M36" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="N36" s="17"/>
+    </row>
+    <row r="37" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A37" s="13">
+        <v>46274</v>
+      </c>
+      <c r="B37" s="14">
+        <v>420</v>
+      </c>
+      <c r="C37" s="14">
+        <v>30</v>
+      </c>
+      <c r="D37" s="14">
+        <v>150</v>
+      </c>
+      <c r="E37" s="14">
+        <v>50</v>
+      </c>
+      <c r="F37" s="14">
+        <v>300</v>
+      </c>
+      <c r="G37" s="14">
+        <v>6</v>
+      </c>
+      <c r="H37" s="14">
+        <v>110</v>
+      </c>
+      <c r="I37" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J36" s="15" t="str">
+        <v>1060</v>
+      </c>
+      <c r="J37" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K36" s="16"/>
-      <c r="L36" s="16"/>
-      <c r="M36" s="16"/>
-      <c r="N36" s="17"/>
-    </row>
-    <row r="37" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A37" s="13"/>
-      <c r="B37" s="14"/>
-      <c r="C37" s="14"/>
-      <c r="D37" s="14"/>
-      <c r="E37" s="14"/>
-      <c r="F37" s="14"/>
-      <c r="G37" s="14"/>
-      <c r="H37" s="14"/>
-      <c r="I37" s="15" t="str">
+        <v>380</v>
+      </c>
+      <c r="K37" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="L37" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M37" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="N37" s="17"/>
+    </row>
+    <row r="38" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A38" s="13">
+        <v>46275</v>
+      </c>
+      <c r="B38" s="14">
+        <v>350</v>
+      </c>
+      <c r="C38" s="14">
+        <v>30</v>
+      </c>
+      <c r="D38" s="14">
+        <v>110</v>
+      </c>
+      <c r="E38" s="14">
+        <v>120</v>
+      </c>
+      <c r="F38" s="14">
+        <v>50</v>
+      </c>
+      <c r="G38" s="14">
+        <v>1</v>
+      </c>
+      <c r="H38" s="14">
+        <v>230</v>
+      </c>
+      <c r="I38" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J37" s="15" t="str">
+        <v>890</v>
+      </c>
+      <c r="J38" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K37" s="16"/>
-      <c r="L37" s="16"/>
-      <c r="M37" s="16"/>
-      <c r="N37" s="17"/>
-    </row>
-    <row r="38" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A38" s="13"/>
-      <c r="B38" s="14"/>
-      <c r="C38" s="14"/>
-      <c r="D38" s="14"/>
-      <c r="E38" s="14"/>
-      <c r="F38" s="14"/>
-      <c r="G38" s="14"/>
-      <c r="H38" s="14"/>
-      <c r="I38" s="15" t="str">
+        <v>550</v>
+      </c>
+      <c r="K38" s="16" t="s">
+        <v>63</v>
+      </c>
+      <c r="L38" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="M38" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="N38" s="17" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="39" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A39" s="13">
+        <v>46276</v>
+      </c>
+      <c r="B39" s="14">
+        <v>510</v>
+      </c>
+      <c r="C39" s="14">
+        <v>20</v>
+      </c>
+      <c r="D39" s="14">
+        <v>200</v>
+      </c>
+      <c r="E39" s="14">
+        <v>20</v>
+      </c>
+      <c r="F39" s="14">
+        <v>300</v>
+      </c>
+      <c r="G39" s="14">
+        <v>6</v>
+      </c>
+      <c r="H39" s="14">
+        <v>50</v>
+      </c>
+      <c r="I39" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J38" s="15" t="str">
+        <v>1100</v>
+      </c>
+      <c r="J39" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K38" s="16"/>
-      <c r="L38" s="16"/>
-      <c r="M38" s="16"/>
-      <c r="N38" s="17"/>
-    </row>
-    <row r="39" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A39" s="13"/>
-      <c r="B39" s="14"/>
-      <c r="C39" s="14"/>
-      <c r="D39" s="14"/>
-      <c r="E39" s="14"/>
-      <c r="F39" s="14"/>
-      <c r="G39" s="14"/>
-      <c r="H39" s="14"/>
-      <c r="I39" s="15" t="str">
+        <v>340</v>
+      </c>
+      <c r="K39" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L39" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="M39" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="N39" s="17"/>
+    </row>
+    <row r="40" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A40" s="13">
+        <v>46277</v>
+      </c>
+      <c r="B40" s="14">
+        <v>500</v>
+      </c>
+      <c r="C40" s="14">
+        <v>15</v>
+      </c>
+      <c r="D40" s="14">
+        <v>160</v>
+      </c>
+      <c r="E40" s="14">
+        <v>30</v>
+      </c>
+      <c r="F40" s="14" t="s">
+        <v>71</v>
+      </c>
+      <c r="G40" s="14" t="s">
+        <v>68</v>
+      </c>
+      <c r="H40" s="14">
+        <v>480</v>
+      </c>
+      <c r="I40" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J39" s="15" t="str">
+        <v>1185</v>
+      </c>
+      <c r="J40" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K39" s="16"/>
-      <c r="L39" s="16"/>
-      <c r="M39" s="16"/>
-      <c r="N39" s="17"/>
-    </row>
-    <row r="40" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A40" s="13"/>
-      <c r="B40" s="14"/>
-      <c r="C40" s="14"/>
-      <c r="D40" s="14"/>
-      <c r="E40" s="14"/>
-      <c r="F40" s="14"/>
-      <c r="G40" s="14"/>
-      <c r="H40" s="14"/>
-      <c r="I40" s="15" t="str">
+        <v>255</v>
+      </c>
+      <c r="K40" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L40" s="16" t="s">
+        <v>64</v>
+      </c>
+      <c r="M40" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="N40" s="17" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="41" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A41" s="13">
+        <v>46278</v>
+      </c>
+      <c r="B41" s="14">
+        <v>530</v>
+      </c>
+      <c r="C41" s="14">
+        <v>10</v>
+      </c>
+      <c r="D41" s="14">
+        <v>190</v>
+      </c>
+      <c r="E41" s="14">
+        <v>50</v>
+      </c>
+      <c r="F41" s="14" t="s">
+        <v>71</v>
+      </c>
+      <c r="G41" s="14" t="s">
+        <v>69</v>
+      </c>
+      <c r="H41" s="14">
+        <v>430</v>
+      </c>
+      <c r="I41" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J40" s="15" t="str">
+        <v>1210</v>
+      </c>
+      <c r="J41" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K40" s="16"/>
-      <c r="L40" s="16"/>
-      <c r="M40" s="16"/>
-      <c r="N40" s="17"/>
-    </row>
-    <row r="41" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A41" s="13"/>
-      <c r="B41" s="14"/>
-      <c r="C41" s="14"/>
-      <c r="D41" s="14"/>
-      <c r="E41" s="14"/>
-      <c r="F41" s="14"/>
-      <c r="G41" s="14"/>
-      <c r="H41" s="14"/>
-      <c r="I41" s="15" t="str">
+        <v>230</v>
+      </c>
+      <c r="K41" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L41" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M41" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N41" s="17" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="42" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A42" s="13">
+        <v>46279</v>
+      </c>
+      <c r="B42" s="14">
+        <v>300</v>
+      </c>
+      <c r="C42" s="14">
+        <v>0</v>
+      </c>
+      <c r="D42" s="14">
+        <v>0</v>
+      </c>
+      <c r="E42" s="14">
+        <v>0</v>
+      </c>
+      <c r="F42" s="14">
+        <v>250</v>
+      </c>
+      <c r="G42" s="14">
+        <v>5</v>
+      </c>
+      <c r="H42" s="14">
+        <v>240</v>
+      </c>
+      <c r="I42" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J41" s="15" t="str">
+        <v>790</v>
+      </c>
+      <c r="J42" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K41" s="16"/>
-      <c r="L41" s="16"/>
-      <c r="M41" s="16"/>
-      <c r="N41" s="17"/>
-    </row>
-    <row r="42" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A42" s="13"/>
-      <c r="B42" s="14"/>
-      <c r="C42" s="14"/>
-      <c r="D42" s="14"/>
-      <c r="E42" s="14"/>
-      <c r="F42" s="14"/>
-      <c r="G42" s="14"/>
-      <c r="H42" s="14"/>
-      <c r="I42" s="15" t="str">
+        <v>650</v>
+      </c>
+      <c r="K42" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L42" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M42" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="N42" s="17" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="43" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A43" s="13">
+        <v>46280</v>
+      </c>
+      <c r="B43" s="14">
+        <v>260</v>
+      </c>
+      <c r="C43" s="14">
+        <v>0</v>
+      </c>
+      <c r="D43" s="14">
+        <v>0</v>
+      </c>
+      <c r="E43" s="14">
+        <v>0</v>
+      </c>
+      <c r="F43" s="14">
+        <v>0</v>
+      </c>
+      <c r="G43" s="14" t="s">
+        <v>71</v>
+      </c>
+      <c r="H43" s="14">
+        <v>250</v>
+      </c>
+      <c r="I43" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J42" s="15" t="str">
+        <v>510</v>
+      </c>
+      <c r="J43" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K42" s="16"/>
-      <c r="L42" s="16"/>
-      <c r="M42" s="16"/>
-      <c r="N42" s="17"/>
-    </row>
-    <row r="43" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A43" s="13"/>
-      <c r="B43" s="14"/>
-      <c r="C43" s="14"/>
-      <c r="D43" s="14"/>
-      <c r="E43" s="14"/>
-      <c r="F43" s="14"/>
-      <c r="G43" s="14"/>
-      <c r="H43" s="14"/>
-      <c r="I43" s="15" t="str">
+        <v>930</v>
+      </c>
+      <c r="K43" s="16" t="s">
+        <v>63</v>
+      </c>
+      <c r="L43" s="16" t="s">
+        <v>64</v>
+      </c>
+      <c r="M43" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="N43" s="17" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="44" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A44" s="13">
+        <v>46281</v>
+      </c>
+      <c r="B44" s="14">
+        <v>450</v>
+      </c>
+      <c r="C44" s="14">
+        <v>0</v>
+      </c>
+      <c r="D44" s="14">
+        <v>0</v>
+      </c>
+      <c r="E44" s="14">
+        <v>0</v>
+      </c>
+      <c r="F44" s="14">
+        <v>0</v>
+      </c>
+      <c r="G44" s="14" t="s">
+        <v>71</v>
+      </c>
+      <c r="H44" s="14">
+        <v>30</v>
+      </c>
+      <c r="I44" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J43" s="15" t="str">
+        <v>480</v>
+      </c>
+      <c r="J44" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K43" s="16"/>
-      <c r="L43" s="16"/>
-      <c r="M43" s="16"/>
-      <c r="N43" s="17"/>
-    </row>
-    <row r="44" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A44" s="13"/>
-      <c r="B44" s="14"/>
-      <c r="C44" s="14"/>
-      <c r="D44" s="14"/>
-      <c r="E44" s="14"/>
-      <c r="F44" s="14"/>
-      <c r="G44" s="14"/>
-      <c r="H44" s="14"/>
-      <c r="I44" s="15" t="str">
+        <v>960</v>
+      </c>
+      <c r="K44" s="16" t="s">
+        <v>63</v>
+      </c>
+      <c r="L44" s="16" t="s">
+        <v>64</v>
+      </c>
+      <c r="M44" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="N44" s="17" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="45" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A45" s="13">
+        <v>46282</v>
+      </c>
+      <c r="B45" s="14">
+        <v>440</v>
+      </c>
+      <c r="C45" s="14">
+        <v>0</v>
+      </c>
+      <c r="D45" s="14">
+        <v>0</v>
+      </c>
+      <c r="E45" s="14">
+        <v>0</v>
+      </c>
+      <c r="F45" s="14">
+        <v>0</v>
+      </c>
+      <c r="G45" s="14" t="s">
+        <v>71</v>
+      </c>
+      <c r="H45" s="14">
+        <v>50</v>
+      </c>
+      <c r="I45" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J44" s="15" t="str">
+        <v>490</v>
+      </c>
+      <c r="J45" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K44" s="16"/>
-      <c r="L44" s="16"/>
-      <c r="M44" s="16"/>
-      <c r="N44" s="17"/>
-    </row>
-    <row r="45" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A45" s="13"/>
-      <c r="B45" s="14"/>
-      <c r="C45" s="14"/>
-      <c r="D45" s="14"/>
-      <c r="E45" s="14"/>
-      <c r="F45" s="14"/>
-      <c r="G45" s="14"/>
-      <c r="H45" s="14"/>
-      <c r="I45" s="15" t="str">
+        <v>950</v>
+      </c>
+      <c r="K45" s="16" t="s">
+        <v>63</v>
+      </c>
+      <c r="L45" s="16" t="s">
+        <v>64</v>
+      </c>
+      <c r="M45" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="N45" s="17" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="46" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A46" s="13">
+        <v>46283</v>
+      </c>
+      <c r="B46" s="14">
+        <v>430</v>
+      </c>
+      <c r="C46" s="14">
+        <v>0</v>
+      </c>
+      <c r="D46" s="14">
+        <v>0</v>
+      </c>
+      <c r="E46" s="14">
+        <v>0</v>
+      </c>
+      <c r="F46" s="14">
+        <v>0</v>
+      </c>
+      <c r="G46" s="14" t="s">
+        <v>71</v>
+      </c>
+      <c r="H46" s="14">
+        <v>50</v>
+      </c>
+      <c r="I46" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J45" s="15" t="str">
+        <v>480</v>
+      </c>
+      <c r="J46" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K45" s="16"/>
-      <c r="L45" s="16"/>
-      <c r="M45" s="16"/>
-      <c r="N45" s="17"/>
-    </row>
-    <row r="46" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A46" s="13"/>
-      <c r="B46" s="14"/>
-      <c r="C46" s="14"/>
-      <c r="D46" s="14"/>
-      <c r="E46" s="14"/>
-      <c r="F46" s="14"/>
-      <c r="G46" s="14"/>
-      <c r="H46" s="14"/>
-      <c r="I46" s="15" t="str">
+        <v>960</v>
+      </c>
+      <c r="K46" s="16" t="s">
+        <v>63</v>
+      </c>
+      <c r="L46" s="16" t="s">
+        <v>64</v>
+      </c>
+      <c r="M46" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N46" s="17" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="47" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A47" s="13">
+        <v>46284</v>
+      </c>
+      <c r="B47" s="14">
+        <v>490</v>
+      </c>
+      <c r="C47" s="14">
+        <v>0</v>
+      </c>
+      <c r="D47" s="14">
+        <v>0</v>
+      </c>
+      <c r="E47" s="14">
+        <v>0</v>
+      </c>
+      <c r="F47" s="14">
+        <v>0</v>
+      </c>
+      <c r="G47" s="14" t="s">
+        <v>68</v>
+      </c>
+      <c r="H47" s="14">
+        <v>240</v>
+      </c>
+      <c r="I47" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J46" s="15" t="str">
+        <v>730</v>
+      </c>
+      <c r="J47" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K46" s="16"/>
-      <c r="L46" s="16"/>
-      <c r="M46" s="16"/>
-      <c r="N46" s="17"/>
-    </row>
-    <row r="47" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A47" s="13"/>
-      <c r="B47" s="14"/>
-      <c r="C47" s="14"/>
-      <c r="D47" s="14"/>
-      <c r="E47" s="14"/>
-      <c r="F47" s="14"/>
-      <c r="G47" s="14"/>
-      <c r="H47" s="14"/>
-      <c r="I47" s="15" t="str">
+        <v>710</v>
+      </c>
+      <c r="K47" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="L47" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M47" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N47" s="17" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="48" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A48" s="13">
+        <v>46285</v>
+      </c>
+      <c r="B48" s="14">
+        <v>480</v>
+      </c>
+      <c r="C48" s="14">
+        <v>0</v>
+      </c>
+      <c r="D48" s="14">
+        <v>0</v>
+      </c>
+      <c r="E48" s="14">
+        <v>0</v>
+      </c>
+      <c r="F48" s="14" t="s">
+        <v>71</v>
+      </c>
+      <c r="G48" s="14" t="s">
+        <v>69</v>
+      </c>
+      <c r="H48" s="14">
+        <v>240</v>
+      </c>
+      <c r="I48" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J47" s="15" t="str">
+        <v>720</v>
+      </c>
+      <c r="J48" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K47" s="16"/>
-      <c r="L47" s="16"/>
-      <c r="M47" s="16"/>
-      <c r="N47" s="17"/>
-    </row>
-    <row r="48" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A48" s="13"/>
-      <c r="B48" s="14"/>
-      <c r="C48" s="14"/>
-      <c r="D48" s="14"/>
-      <c r="E48" s="14"/>
-      <c r="F48" s="14"/>
-      <c r="G48" s="14"/>
-      <c r="H48" s="14"/>
-      <c r="I48" s="15" t="str">
+        <v>720</v>
+      </c>
+      <c r="K48" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="L48" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="M48" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="N48" s="17" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="49" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A49" s="13">
+        <v>46286</v>
+      </c>
+      <c r="B49" s="14">
+        <v>430</v>
+      </c>
+      <c r="C49" s="14">
+        <v>0</v>
+      </c>
+      <c r="D49" s="14">
+        <v>120</v>
+      </c>
+      <c r="E49" s="14">
+        <v>50</v>
+      </c>
+      <c r="F49" s="14">
+        <v>250</v>
+      </c>
+      <c r="G49" s="14">
+        <v>6</v>
+      </c>
+      <c r="H49" s="14">
+        <v>60</v>
+      </c>
+      <c r="I49" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J48" s="15" t="str">
+        <v>910</v>
+      </c>
+      <c r="J49" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K48" s="16"/>
-      <c r="L48" s="16"/>
-      <c r="M48" s="16"/>
-      <c r="N48" s="17"/>
-    </row>
-    <row r="49" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A49" s="13"/>
-      <c r="B49" s="14"/>
-      <c r="C49" s="14"/>
-      <c r="D49" s="14"/>
-      <c r="E49" s="14"/>
-      <c r="F49" s="14"/>
-      <c r="G49" s="14"/>
-      <c r="H49" s="14"/>
-      <c r="I49" s="15" t="str">
+        <v>530</v>
+      </c>
+      <c r="K49" s="16" t="s">
+        <v>60</v>
+      </c>
+      <c r="L49" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="M49" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="N49" s="17" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="50" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A50" s="13">
+        <v>46287</v>
+      </c>
+      <c r="B50" s="14">
+        <v>350</v>
+      </c>
+      <c r="C50" s="14">
+        <v>30</v>
+      </c>
+      <c r="D50" s="14">
+        <v>290</v>
+      </c>
+      <c r="E50" s="14">
+        <v>0</v>
+      </c>
+      <c r="F50" s="14">
+        <v>350</v>
+      </c>
+      <c r="G50" s="14">
+        <v>7</v>
+      </c>
+      <c r="H50" s="14">
+        <v>50</v>
+      </c>
+      <c r="I50" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J49" s="15" t="str">
+        <v>1070</v>
+      </c>
+      <c r="J50" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K49" s="16"/>
-      <c r="L49" s="16"/>
-      <c r="M49" s="16"/>
-      <c r="N49" s="17"/>
-    </row>
-    <row r="50" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A50" s="13"/>
-      <c r="B50" s="14"/>
-      <c r="C50" s="14"/>
-      <c r="D50" s="14"/>
-      <c r="E50" s="14"/>
-      <c r="F50" s="14"/>
-      <c r="G50" s="14"/>
-      <c r="H50" s="14"/>
-      <c r="I50" s="15" t="str">
+        <v>370</v>
+      </c>
+      <c r="K50" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="L50" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="M50" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N50" s="17" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="51" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A51" s="13">
+        <v>46288</v>
+      </c>
+      <c r="B51" s="14">
+        <v>360</v>
+      </c>
+      <c r="C51" s="14">
+        <v>20</v>
+      </c>
+      <c r="D51" s="14">
+        <v>120</v>
+      </c>
+      <c r="E51" s="14">
+        <v>50</v>
+      </c>
+      <c r="F51" s="14">
+        <v>300</v>
+      </c>
+      <c r="G51" s="14">
+        <v>7</v>
+      </c>
+      <c r="H51" s="14">
+        <v>200</v>
+      </c>
+      <c r="I51" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J50" s="15" t="str">
+        <v>1050</v>
+      </c>
+      <c r="J51" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K50" s="16"/>
-      <c r="L50" s="16"/>
-      <c r="M50" s="16"/>
-      <c r="N50" s="17"/>
-    </row>
-    <row r="51" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A51" s="13"/>
-      <c r="B51" s="14"/>
-      <c r="C51" s="14"/>
-      <c r="D51" s="14"/>
-      <c r="E51" s="14"/>
-      <c r="F51" s="14"/>
-      <c r="G51" s="14"/>
-      <c r="H51" s="14"/>
-      <c r="I51" s="15" t="str">
+        <v>390</v>
+      </c>
+      <c r="K51" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L51" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M51" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N51" s="17" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="52" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A52" s="13">
+        <v>46289</v>
+      </c>
+      <c r="B52" s="14">
+        <v>480</v>
+      </c>
+      <c r="C52" s="14">
+        <v>10</v>
+      </c>
+      <c r="D52" s="14">
+        <v>95</v>
+      </c>
+      <c r="E52" s="14">
+        <v>120</v>
+      </c>
+      <c r="F52" s="14">
+        <v>100</v>
+      </c>
+      <c r="G52" s="14">
+        <v>2</v>
+      </c>
+      <c r="H52" s="14">
+        <v>240</v>
+      </c>
+      <c r="I52" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J51" s="15" t="str">
+        <v>1045</v>
+      </c>
+      <c r="J52" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K51" s="16"/>
-      <c r="L51" s="16"/>
-      <c r="M51" s="16"/>
-      <c r="N51" s="17"/>
-    </row>
-    <row r="52" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A52" s="13"/>
-      <c r="B52" s="14"/>
-      <c r="C52" s="14"/>
-      <c r="D52" s="14"/>
-      <c r="E52" s="14"/>
-      <c r="F52" s="14"/>
-      <c r="G52" s="14"/>
-      <c r="H52" s="14"/>
-      <c r="I52" s="15" t="str">
+        <v>395</v>
+      </c>
+      <c r="K52" s="16" t="s">
+        <v>63</v>
+      </c>
+      <c r="L52" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M52" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="N52" s="17" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="53" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A53" s="13">
+        <v>46290</v>
+      </c>
+      <c r="B53" s="14">
+        <v>230</v>
+      </c>
+      <c r="C53" s="14">
+        <v>20</v>
+      </c>
+      <c r="D53" s="14">
+        <v>60</v>
+      </c>
+      <c r="E53" s="14">
+        <v>150</v>
+      </c>
+      <c r="F53" s="14">
+        <v>300</v>
+      </c>
+      <c r="G53" s="14">
+        <v>6</v>
+      </c>
+      <c r="H53" s="14">
+        <v>50</v>
+      </c>
+      <c r="I53" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J52" s="15" t="str">
+        <v>810</v>
+      </c>
+      <c r="J53" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K52" s="16"/>
-      <c r="L52" s="16"/>
-      <c r="M52" s="16"/>
-      <c r="N52" s="17"/>
-    </row>
-    <row r="53" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A53" s="13"/>
-      <c r="B53" s="14"/>
-      <c r="C53" s="14"/>
-      <c r="D53" s="14"/>
-      <c r="E53" s="14"/>
-      <c r="F53" s="14"/>
-      <c r="G53" s="14"/>
-      <c r="H53" s="14"/>
-      <c r="I53" s="15" t="str">
+        <v>630</v>
+      </c>
+      <c r="K53" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L53" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="M53" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N53" s="17"/>
+    </row>
+    <row r="54" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A54" s="13">
+        <v>46291</v>
+      </c>
+      <c r="B54" s="14">
+        <v>350</v>
+      </c>
+      <c r="C54" s="14">
+        <v>60</v>
+      </c>
+      <c r="D54" s="14">
+        <v>50</v>
+      </c>
+      <c r="E54" s="14">
+        <v>130</v>
+      </c>
+      <c r="F54" s="14">
+        <v>0</v>
+      </c>
+      <c r="G54" s="14" t="s">
+        <v>68</v>
+      </c>
+      <c r="H54" s="14">
+        <v>240</v>
+      </c>
+      <c r="I54" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J53" s="15" t="str">
+        <v>830</v>
+      </c>
+      <c r="J54" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K53" s="16"/>
-      <c r="L53" s="16"/>
-      <c r="M53" s="16"/>
-      <c r="N53" s="17"/>
-    </row>
-    <row r="54" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A54" s="13"/>
-      <c r="B54" s="14"/>
-      <c r="C54" s="14"/>
-      <c r="D54" s="14"/>
-      <c r="E54" s="14"/>
-      <c r="F54" s="14"/>
-      <c r="G54" s="14"/>
-      <c r="H54" s="14"/>
-      <c r="I54" s="15" t="str">
+        <v>610</v>
+      </c>
+      <c r="K54" s="16" t="s">
+        <v>63</v>
+      </c>
+      <c r="L54" s="16" t="s">
+        <v>72</v>
+      </c>
+      <c r="M54" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N54" s="17"/>
+    </row>
+    <row r="55" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A55" s="13">
+        <v>46292</v>
+      </c>
+      <c r="B55" s="14">
+        <v>490</v>
+      </c>
+      <c r="C55" s="14">
+        <v>30</v>
+      </c>
+      <c r="D55" s="14">
+        <v>90</v>
+      </c>
+      <c r="E55" s="14">
+        <v>50</v>
+      </c>
+      <c r="F55" s="14">
+        <v>0</v>
+      </c>
+      <c r="G55" s="14" t="s">
+        <v>69</v>
+      </c>
+      <c r="H55" s="14">
+        <v>240</v>
+      </c>
+      <c r="I55" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J54" s="15" t="str">
+        <v>900</v>
+      </c>
+      <c r="J55" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K54" s="16"/>
-      <c r="L54" s="16"/>
-      <c r="M54" s="16"/>
-      <c r="N54" s="17"/>
-    </row>
-    <row r="55" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A55" s="13"/>
-      <c r="B55" s="14"/>
-      <c r="C55" s="14"/>
-      <c r="D55" s="14"/>
-      <c r="E55" s="14"/>
-      <c r="F55" s="14"/>
-      <c r="G55" s="14"/>
-      <c r="H55" s="14"/>
-      <c r="I55" s="15" t="str">
+        <v>540</v>
+      </c>
+      <c r="K55" s="16" t="s">
+        <v>63</v>
+      </c>
+      <c r="L55" s="16" t="s">
+        <v>72</v>
+      </c>
+      <c r="M55" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="N55" s="17" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="56" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A56" s="13">
+        <v>46293</v>
+      </c>
+      <c r="B56" s="14">
+        <v>340</v>
+      </c>
+      <c r="C56" s="14">
+        <v>20</v>
+      </c>
+      <c r="D56" s="14">
+        <v>0</v>
+      </c>
+      <c r="E56" s="14">
+        <v>0</v>
+      </c>
+      <c r="F56" s="14">
+        <v>0</v>
+      </c>
+      <c r="G56" s="14">
+        <v>0</v>
+      </c>
+      <c r="H56" s="14">
+        <v>110</v>
+      </c>
+      <c r="I56" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J55" s="15" t="str">
+        <v>470</v>
+      </c>
+      <c r="J56" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K55" s="16"/>
-      <c r="L55" s="16"/>
-      <c r="M55" s="16"/>
-      <c r="N55" s="17"/>
-    </row>
-    <row r="56" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A56" s="13"/>
-      <c r="B56" s="14"/>
-      <c r="C56" s="14"/>
-      <c r="D56" s="14"/>
-      <c r="E56" s="14"/>
-      <c r="F56" s="14"/>
-      <c r="G56" s="14"/>
-      <c r="H56" s="14"/>
-      <c r="I56" s="15" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J56" s="15" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K56" s="16"/>
-      <c r="L56" s="16"/>
-      <c r="M56" s="16"/>
-      <c r="N56" s="17"/>
+        <v>970</v>
+      </c>
+      <c r="K56" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="L56" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="M56" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N56" s="17" t="s">
+        <v>102</v>
+      </c>
     </row>
     <row r="57" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A57" s="13"/>
+      <c r="A57" s="13">
+        <v>46294</v>
+      </c>
       <c r="B57" s="14"/>
       <c r="C57" s="14"/>
       <c r="D57" s="14"/>
       <c r="E57" s="14"/>
-      <c r="F57" s="14"/>
-      <c r="G57" s="14"/>
+      <c r="F57" s="14">
+        <v>0</v>
+      </c>
+      <c r="G57" s="14">
+        <v>0</v>
+      </c>
       <c r="H57" s="14"/>
       <c r="I57" s="15" t="str">
         <f t="shared" si="0"/>
@@ -2416,13 +3471,19 @@
       <c r="N57" s="17"/>
     </row>
     <row r="58" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A58" s="13"/>
+      <c r="A58" s="13">
+        <v>46295</v>
+      </c>
       <c r="B58" s="14"/>
       <c r="C58" s="14"/>
       <c r="D58" s="14"/>
       <c r="E58" s="14"/>
-      <c r="F58" s="14"/>
-      <c r="G58" s="14"/>
+      <c r="F58" s="14">
+        <v>0</v>
+      </c>
+      <c r="G58" s="14">
+        <v>0</v>
+      </c>
       <c r="H58" s="14"/>
       <c r="I58" s="15" t="str">
         <f t="shared" si="0"/>
@@ -2438,13 +3499,19 @@
       <c r="N58" s="17"/>
     </row>
     <row r="59" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A59" s="13"/>
+      <c r="A59" s="13">
+        <v>46296</v>
+      </c>
       <c r="B59" s="14"/>
       <c r="C59" s="14"/>
       <c r="D59" s="14"/>
       <c r="E59" s="14"/>
-      <c r="F59" s="14"/>
-      <c r="G59" s="14"/>
+      <c r="F59" s="14">
+        <v>0</v>
+      </c>
+      <c r="G59" s="14">
+        <v>0</v>
+      </c>
       <c r="H59" s="14"/>
       <c r="I59" s="15" t="str">
         <f t="shared" si="0"/>
@@ -2460,13 +3527,19 @@
       <c r="N59" s="17"/>
     </row>
     <row r="60" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A60" s="13"/>
+      <c r="A60" s="13">
+        <v>46297</v>
+      </c>
       <c r="B60" s="14"/>
       <c r="C60" s="14"/>
       <c r="D60" s="14"/>
       <c r="E60" s="14"/>
-      <c r="F60" s="14"/>
-      <c r="G60" s="14"/>
+      <c r="F60" s="14">
+        <v>0</v>
+      </c>
+      <c r="G60" s="14">
+        <v>0</v>
+      </c>
       <c r="H60" s="14"/>
       <c r="I60" s="15" t="str">
         <f t="shared" si="0"/>
@@ -2482,13 +3555,19 @@
       <c r="N60" s="17"/>
     </row>
     <row r="61" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A61" s="13"/>
+      <c r="A61" s="13">
+        <v>46298</v>
+      </c>
       <c r="B61" s="14"/>
       <c r="C61" s="14"/>
       <c r="D61" s="14"/>
       <c r="E61" s="14"/>
-      <c r="F61" s="14"/>
-      <c r="G61" s="14"/>
+      <c r="F61" s="14">
+        <v>0</v>
+      </c>
+      <c r="G61" s="14">
+        <v>0</v>
+      </c>
       <c r="H61" s="14"/>
       <c r="I61" s="15" t="str">
         <f t="shared" si="0"/>
@@ -2509,8 +3588,12 @@
       <c r="C62" s="14"/>
       <c r="D62" s="14"/>
       <c r="E62" s="14"/>
-      <c r="F62" s="14"/>
-      <c r="G62" s="14"/>
+      <c r="F62" s="14">
+        <v>0</v>
+      </c>
+      <c r="G62" s="14">
+        <v>0</v>
+      </c>
       <c r="H62" s="14"/>
       <c r="I62" s="15" t="str">
         <f t="shared" si="0"/>
@@ -2531,8 +3614,12 @@
       <c r="C63" s="14"/>
       <c r="D63" s="14"/>
       <c r="E63" s="14"/>
-      <c r="F63" s="14"/>
-      <c r="G63" s="14"/>
+      <c r="F63" s="14">
+        <v>0</v>
+      </c>
+      <c r="G63" s="14">
+        <v>0</v>
+      </c>
       <c r="H63" s="14"/>
       <c r="I63" s="15" t="str">
         <f t="shared" si="0"/>
@@ -2553,8 +3640,12 @@
       <c r="C64" s="14"/>
       <c r="D64" s="14"/>
       <c r="E64" s="14"/>
-      <c r="F64" s="14"/>
-      <c r="G64" s="14"/>
+      <c r="F64" s="14">
+        <v>0</v>
+      </c>
+      <c r="G64" s="14">
+        <v>0</v>
+      </c>
       <c r="H64" s="14"/>
       <c r="I64" s="15" t="str">
         <f t="shared" si="0"/>
@@ -2575,8 +3666,12 @@
       <c r="C65" s="14"/>
       <c r="D65" s="14"/>
       <c r="E65" s="14"/>
-      <c r="F65" s="14"/>
-      <c r="G65" s="14"/>
+      <c r="F65" s="14">
+        <v>0</v>
+      </c>
+      <c r="G65" s="14">
+        <v>0</v>
+      </c>
       <c r="H65" s="14"/>
       <c r="I65" s="15" t="str">
         <f t="shared" si="0"/>

</xml_diff>